<commit_message>
klote null melding voor de datatable
</commit_message>
<xml_diff>
--- a/Data/Output/CandidateList.xlsx
+++ b/Data/Output/CandidateList.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <x:si>
     <x:t>Name Candidate</x:t>
   </x:si>
@@ -26,6 +26,9 @@
   </x:si>
   <x:si>
     <x:t>Email</x:t>
+  </x:si>
+  <x:si>
+    <x:t>text</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -393,7 +396,11 @@
         <x:v>3</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" spans="1:4"/>
+    <x:row r="2" spans="1:4">
+      <x:c r="A2" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>